<commit_message>
Correct tracker: ads went live Oct 6, US$1.87 spent and 1 message so far
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SDEXtRNKXxCcmXTs5yLNBs
</commit_message>
<xml_diff>
--- a/ads-budget-tracker.xlsx
+++ b/ads-budget-tracker.xlsx
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNT('Daily Ads'!$B$5:$B$93)</f>
+        <f>COUNT('Daily Ads'!$B$5:$B$91)</f>
         <v/>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>'Daily Ads'!$B$94</f>
+        <f>'Daily Ads'!$B$92</f>
         <v/>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>IFERROR('Daily Ads'!$B$94/B5,0)</f>
+        <f>IFERROR('Daily Ads'!$B$92/B5,0)</f>
         <v/>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>Settings!$B$6-SUMIFS('Daily Ads'!$B$5:$B$93,'Daily Ads'!$A$5:$A$93,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'Daily Ads'!$A$5:$A$93,"&lt;="&amp;EOMONTH(TODAY(),0))</f>
+        <f>Settings!$B$6-SUMIFS('Daily Ads'!$B$5:$B$91,'Daily Ads'!$A$5:$A$91,"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),'Daily Ads'!$A$5:$A$91,"&lt;="&amp;EOMONTH(TODAY(),0))</f>
         <v/>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>'Daily Ads'!$E$94</f>
+        <f>'Daily Ads'!$E$92</f>
         <v/>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1199,11 +1199,11 @@
         </is>
       </c>
       <c r="B11" s="19" t="n">
-        <v>46299</v>
+        <v>46301</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>4 days run as of Wed 7 Oct 2026.</t>
+          <t>First ad went live about 12pm on Tue 6 Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I94"/>
+  <dimension ref="A1:I92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1328,14 +1328,16 @@
     </row>
     <row r="5">
       <c r="A5" s="22" t="n">
-        <v>46299</v>
+        <v>46301</v>
       </c>
       <c r="B5" s="23" t="n">
-        <v>5</v>
+        <v>1.87</v>
       </c>
       <c r="C5" s="24" t="n"/>
       <c r="D5" s="24" t="n"/>
-      <c r="E5" s="24" t="n"/>
+      <c r="E5" s="24" t="n">
+        <v>1</v>
+      </c>
       <c r="F5" s="25">
         <f>IF(OR(B5="",E5="",E5=0),"",B5/E5)</f>
         <v/>
@@ -1350,17 +1352,15 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>From you: US$5/day</t>
+          <t>From you: US$1.87 spent and 1 message since launch (~12pm Oct 6) - split by day from Ads Manager if you like</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="B6" s="23" t="n">
-        <v>5</v>
-      </c>
+        <v>46302</v>
+      </c>
+      <c r="B6" s="23" t="n"/>
       <c r="C6" s="24" t="n"/>
       <c r="D6" s="24" t="n"/>
       <c r="E6" s="24" t="n"/>
@@ -1376,19 +1376,13 @@
         <f>IF(B6="","",SUM($B$5:B6))</f>
         <v/>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>From you: US$5/day</t>
-        </is>
-      </c>
+      <c r="I6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="22" t="n">
-        <v>46301</v>
-      </c>
-      <c r="B7" s="23" t="n">
-        <v>5</v>
-      </c>
+        <v>46303</v>
+      </c>
+      <c r="B7" s="23" t="n"/>
       <c r="C7" s="24" t="n"/>
       <c r="D7" s="24" t="n"/>
       <c r="E7" s="24" t="n"/>
@@ -1404,19 +1398,13 @@
         <f>IF(B7="","",SUM($B$5:B7))</f>
         <v/>
       </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>From you: US$5/day</t>
-        </is>
-      </c>
+      <c r="I7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="22" t="n">
-        <v>46302</v>
-      </c>
-      <c r="B8" s="23" t="n">
-        <v>5</v>
-      </c>
+        <v>46304</v>
+      </c>
+      <c r="B8" s="23" t="n"/>
       <c r="C8" s="24" t="n"/>
       <c r="D8" s="24" t="n"/>
       <c r="E8" s="24" t="n"/>
@@ -1432,15 +1420,11 @@
         <f>IF(B8="","",SUM($B$5:B8))</f>
         <v/>
       </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>From you: US$5/day</t>
-        </is>
-      </c>
+      <c r="I8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="22" t="n">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="B9" s="23" t="n"/>
       <c r="C9" s="24" t="n"/>
@@ -1462,7 +1446,7 @@
     </row>
     <row r="10">
       <c r="A10" s="22" t="n">
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="B10" s="23" t="n"/>
       <c r="C10" s="24" t="n"/>
@@ -1484,7 +1468,7 @@
     </row>
     <row r="11">
       <c r="A11" s="22" t="n">
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="B11" s="23" t="n"/>
       <c r="C11" s="24" t="n"/>
@@ -1506,7 +1490,7 @@
     </row>
     <row r="12">
       <c r="A12" s="22" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B12" s="23" t="n"/>
       <c r="C12" s="24" t="n"/>
@@ -1528,7 +1512,7 @@
     </row>
     <row r="13">
       <c r="A13" s="22" t="n">
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="B13" s="23" t="n"/>
       <c r="C13" s="24" t="n"/>
@@ -1550,7 +1534,7 @@
     </row>
     <row r="14">
       <c r="A14" s="22" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="B14" s="23" t="n"/>
       <c r="C14" s="24" t="n"/>
@@ -1572,7 +1556,7 @@
     </row>
     <row r="15">
       <c r="A15" s="22" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="B15" s="23" t="n"/>
       <c r="C15" s="24" t="n"/>
@@ -1594,7 +1578,7 @@
     </row>
     <row r="16">
       <c r="A16" s="22" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="B16" s="23" t="n"/>
       <c r="C16" s="24" t="n"/>
@@ -1616,7 +1600,7 @@
     </row>
     <row r="17">
       <c r="A17" s="22" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
       <c r="B17" s="23" t="n"/>
       <c r="C17" s="24" t="n"/>
@@ -1638,7 +1622,7 @@
     </row>
     <row r="18">
       <c r="A18" s="22" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B18" s="23" t="n"/>
       <c r="C18" s="24" t="n"/>
@@ -1660,7 +1644,7 @@
     </row>
     <row r="19">
       <c r="A19" s="22" t="n">
-        <v>46313</v>
+        <v>46315</v>
       </c>
       <c r="B19" s="23" t="n"/>
       <c r="C19" s="24" t="n"/>
@@ -1682,7 +1666,7 @@
     </row>
     <row r="20">
       <c r="A20" s="22" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="B20" s="23" t="n"/>
       <c r="C20" s="24" t="n"/>
@@ -1704,7 +1688,7 @@
     </row>
     <row r="21">
       <c r="A21" s="22" t="n">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="B21" s="23" t="n"/>
       <c r="C21" s="24" t="n"/>
@@ -1726,7 +1710,7 @@
     </row>
     <row r="22">
       <c r="A22" s="22" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="B22" s="23" t="n"/>
       <c r="C22" s="24" t="n"/>
@@ -1748,7 +1732,7 @@
     </row>
     <row r="23">
       <c r="A23" s="22" t="n">
-        <v>46317</v>
+        <v>46319</v>
       </c>
       <c r="B23" s="23" t="n"/>
       <c r="C23" s="24" t="n"/>
@@ -1770,7 +1754,7 @@
     </row>
     <row r="24">
       <c r="A24" s="22" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
       <c r="B24" s="23" t="n"/>
       <c r="C24" s="24" t="n"/>
@@ -1792,7 +1776,7 @@
     </row>
     <row r="25">
       <c r="A25" s="22" t="n">
-        <v>46319</v>
+        <v>46321</v>
       </c>
       <c r="B25" s="23" t="n"/>
       <c r="C25" s="24" t="n"/>
@@ -1814,7 +1798,7 @@
     </row>
     <row r="26">
       <c r="A26" s="22" t="n">
-        <v>46320</v>
+        <v>46322</v>
       </c>
       <c r="B26" s="23" t="n"/>
       <c r="C26" s="24" t="n"/>
@@ -1836,7 +1820,7 @@
     </row>
     <row r="27">
       <c r="A27" s="22" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="B27" s="23" t="n"/>
       <c r="C27" s="24" t="n"/>
@@ -1858,7 +1842,7 @@
     </row>
     <row r="28">
       <c r="A28" s="22" t="n">
-        <v>46322</v>
+        <v>46324</v>
       </c>
       <c r="B28" s="23" t="n"/>
       <c r="C28" s="24" t="n"/>
@@ -1880,7 +1864,7 @@
     </row>
     <row r="29">
       <c r="A29" s="22" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
       <c r="B29" s="23" t="n"/>
       <c r="C29" s="24" t="n"/>
@@ -1902,7 +1886,7 @@
     </row>
     <row r="30">
       <c r="A30" s="22" t="n">
-        <v>46324</v>
+        <v>46326</v>
       </c>
       <c r="B30" s="23" t="n"/>
       <c r="C30" s="24" t="n"/>
@@ -1924,7 +1908,7 @@
     </row>
     <row r="31">
       <c r="A31" s="22" t="n">
-        <v>46325</v>
+        <v>46327</v>
       </c>
       <c r="B31" s="23" t="n"/>
       <c r="C31" s="24" t="n"/>
@@ -1946,7 +1930,7 @@
     </row>
     <row r="32">
       <c r="A32" s="22" t="n">
-        <v>46326</v>
+        <v>46328</v>
       </c>
       <c r="B32" s="23" t="n"/>
       <c r="C32" s="24" t="n"/>
@@ -1968,7 +1952,7 @@
     </row>
     <row r="33">
       <c r="A33" s="22" t="n">
-        <v>46327</v>
+        <v>46329</v>
       </c>
       <c r="B33" s="23" t="n"/>
       <c r="C33" s="24" t="n"/>
@@ -1990,7 +1974,7 @@
     </row>
     <row r="34">
       <c r="A34" s="22" t="n">
-        <v>46328</v>
+        <v>46330</v>
       </c>
       <c r="B34" s="23" t="n"/>
       <c r="C34" s="24" t="n"/>
@@ -2012,7 +1996,7 @@
     </row>
     <row r="35">
       <c r="A35" s="22" t="n">
-        <v>46329</v>
+        <v>46331</v>
       </c>
       <c r="B35" s="23" t="n"/>
       <c r="C35" s="24" t="n"/>
@@ -2034,7 +2018,7 @@
     </row>
     <row r="36">
       <c r="A36" s="22" t="n">
-        <v>46330</v>
+        <v>46332</v>
       </c>
       <c r="B36" s="23" t="n"/>
       <c r="C36" s="24" t="n"/>
@@ -2056,7 +2040,7 @@
     </row>
     <row r="37">
       <c r="A37" s="22" t="n">
-        <v>46331</v>
+        <v>46333</v>
       </c>
       <c r="B37" s="23" t="n"/>
       <c r="C37" s="24" t="n"/>
@@ -2078,7 +2062,7 @@
     </row>
     <row r="38">
       <c r="A38" s="22" t="n">
-        <v>46332</v>
+        <v>46334</v>
       </c>
       <c r="B38" s="23" t="n"/>
       <c r="C38" s="24" t="n"/>
@@ -2100,7 +2084,7 @@
     </row>
     <row r="39">
       <c r="A39" s="22" t="n">
-        <v>46333</v>
+        <v>46335</v>
       </c>
       <c r="B39" s="23" t="n"/>
       <c r="C39" s="24" t="n"/>
@@ -2122,7 +2106,7 @@
     </row>
     <row r="40">
       <c r="A40" s="22" t="n">
-        <v>46334</v>
+        <v>46336</v>
       </c>
       <c r="B40" s="23" t="n"/>
       <c r="C40" s="24" t="n"/>
@@ -2144,7 +2128,7 @@
     </row>
     <row r="41">
       <c r="A41" s="22" t="n">
-        <v>46335</v>
+        <v>46337</v>
       </c>
       <c r="B41" s="23" t="n"/>
       <c r="C41" s="24" t="n"/>
@@ -2166,7 +2150,7 @@
     </row>
     <row r="42">
       <c r="A42" s="22" t="n">
-        <v>46336</v>
+        <v>46338</v>
       </c>
       <c r="B42" s="23" t="n"/>
       <c r="C42" s="24" t="n"/>
@@ -2188,7 +2172,7 @@
     </row>
     <row r="43">
       <c r="A43" s="22" t="n">
-        <v>46337</v>
+        <v>46339</v>
       </c>
       <c r="B43" s="23" t="n"/>
       <c r="C43" s="24" t="n"/>
@@ -2210,7 +2194,7 @@
     </row>
     <row r="44">
       <c r="A44" s="22" t="n">
-        <v>46338</v>
+        <v>46340</v>
       </c>
       <c r="B44" s="23" t="n"/>
       <c r="C44" s="24" t="n"/>
@@ -2232,7 +2216,7 @@
     </row>
     <row r="45">
       <c r="A45" s="22" t="n">
-        <v>46339</v>
+        <v>46341</v>
       </c>
       <c r="B45" s="23" t="n"/>
       <c r="C45" s="24" t="n"/>
@@ -2254,7 +2238,7 @@
     </row>
     <row r="46">
       <c r="A46" s="22" t="n">
-        <v>46340</v>
+        <v>46342</v>
       </c>
       <c r="B46" s="23" t="n"/>
       <c r="C46" s="24" t="n"/>
@@ -2276,7 +2260,7 @@
     </row>
     <row r="47">
       <c r="A47" s="22" t="n">
-        <v>46341</v>
+        <v>46343</v>
       </c>
       <c r="B47" s="23" t="n"/>
       <c r="C47" s="24" t="n"/>
@@ -2298,7 +2282,7 @@
     </row>
     <row r="48">
       <c r="A48" s="22" t="n">
-        <v>46342</v>
+        <v>46344</v>
       </c>
       <c r="B48" s="23" t="n"/>
       <c r="C48" s="24" t="n"/>
@@ -2320,7 +2304,7 @@
     </row>
     <row r="49">
       <c r="A49" s="22" t="n">
-        <v>46343</v>
+        <v>46345</v>
       </c>
       <c r="B49" s="23" t="n"/>
       <c r="C49" s="24" t="n"/>
@@ -2342,7 +2326,7 @@
     </row>
     <row r="50">
       <c r="A50" s="22" t="n">
-        <v>46344</v>
+        <v>46346</v>
       </c>
       <c r="B50" s="23" t="n"/>
       <c r="C50" s="24" t="n"/>
@@ -2364,7 +2348,7 @@
     </row>
     <row r="51">
       <c r="A51" s="22" t="n">
-        <v>46345</v>
+        <v>46347</v>
       </c>
       <c r="B51" s="23" t="n"/>
       <c r="C51" s="24" t="n"/>
@@ -2386,7 +2370,7 @@
     </row>
     <row r="52">
       <c r="A52" s="22" t="n">
-        <v>46346</v>
+        <v>46348</v>
       </c>
       <c r="B52" s="23" t="n"/>
       <c r="C52" s="24" t="n"/>
@@ -2408,7 +2392,7 @@
     </row>
     <row r="53">
       <c r="A53" s="22" t="n">
-        <v>46347</v>
+        <v>46349</v>
       </c>
       <c r="B53" s="23" t="n"/>
       <c r="C53" s="24" t="n"/>
@@ -2430,7 +2414,7 @@
     </row>
     <row r="54">
       <c r="A54" s="22" t="n">
-        <v>46348</v>
+        <v>46350</v>
       </c>
       <c r="B54" s="23" t="n"/>
       <c r="C54" s="24" t="n"/>
@@ -2452,7 +2436,7 @@
     </row>
     <row r="55">
       <c r="A55" s="22" t="n">
-        <v>46349</v>
+        <v>46351</v>
       </c>
       <c r="B55" s="23" t="n"/>
       <c r="C55" s="24" t="n"/>
@@ -2474,7 +2458,7 @@
     </row>
     <row r="56">
       <c r="A56" s="22" t="n">
-        <v>46350</v>
+        <v>46352</v>
       </c>
       <c r="B56" s="23" t="n"/>
       <c r="C56" s="24" t="n"/>
@@ -2496,7 +2480,7 @@
     </row>
     <row r="57">
       <c r="A57" s="22" t="n">
-        <v>46351</v>
+        <v>46353</v>
       </c>
       <c r="B57" s="23" t="n"/>
       <c r="C57" s="24" t="n"/>
@@ -2518,7 +2502,7 @@
     </row>
     <row r="58">
       <c r="A58" s="22" t="n">
-        <v>46352</v>
+        <v>46354</v>
       </c>
       <c r="B58" s="23" t="n"/>
       <c r="C58" s="24" t="n"/>
@@ -2540,7 +2524,7 @@
     </row>
     <row r="59">
       <c r="A59" s="22" t="n">
-        <v>46353</v>
+        <v>46355</v>
       </c>
       <c r="B59" s="23" t="n"/>
       <c r="C59" s="24" t="n"/>
@@ -2562,7 +2546,7 @@
     </row>
     <row r="60">
       <c r="A60" s="22" t="n">
-        <v>46354</v>
+        <v>46356</v>
       </c>
       <c r="B60" s="23" t="n"/>
       <c r="C60" s="24" t="n"/>
@@ -2584,7 +2568,7 @@
     </row>
     <row r="61">
       <c r="A61" s="22" t="n">
-        <v>46355</v>
+        <v>46357</v>
       </c>
       <c r="B61" s="23" t="n"/>
       <c r="C61" s="24" t="n"/>
@@ -2606,7 +2590,7 @@
     </row>
     <row r="62">
       <c r="A62" s="22" t="n">
-        <v>46356</v>
+        <v>46358</v>
       </c>
       <c r="B62" s="23" t="n"/>
       <c r="C62" s="24" t="n"/>
@@ -2628,7 +2612,7 @@
     </row>
     <row r="63">
       <c r="A63" s="22" t="n">
-        <v>46357</v>
+        <v>46359</v>
       </c>
       <c r="B63" s="23" t="n"/>
       <c r="C63" s="24" t="n"/>
@@ -2650,7 +2634,7 @@
     </row>
     <row r="64">
       <c r="A64" s="22" t="n">
-        <v>46358</v>
+        <v>46360</v>
       </c>
       <c r="B64" s="23" t="n"/>
       <c r="C64" s="24" t="n"/>
@@ -2672,7 +2656,7 @@
     </row>
     <row r="65">
       <c r="A65" s="22" t="n">
-        <v>46359</v>
+        <v>46361</v>
       </c>
       <c r="B65" s="23" t="n"/>
       <c r="C65" s="24" t="n"/>
@@ -2694,7 +2678,7 @@
     </row>
     <row r="66">
       <c r="A66" s="22" t="n">
-        <v>46360</v>
+        <v>46362</v>
       </c>
       <c r="B66" s="23" t="n"/>
       <c r="C66" s="24" t="n"/>
@@ -2716,7 +2700,7 @@
     </row>
     <row r="67">
       <c r="A67" s="22" t="n">
-        <v>46361</v>
+        <v>46363</v>
       </c>
       <c r="B67" s="23" t="n"/>
       <c r="C67" s="24" t="n"/>
@@ -2738,7 +2722,7 @@
     </row>
     <row r="68">
       <c r="A68" s="22" t="n">
-        <v>46362</v>
+        <v>46364</v>
       </c>
       <c r="B68" s="23" t="n"/>
       <c r="C68" s="24" t="n"/>
@@ -2760,7 +2744,7 @@
     </row>
     <row r="69">
       <c r="A69" s="22" t="n">
-        <v>46363</v>
+        <v>46365</v>
       </c>
       <c r="B69" s="23" t="n"/>
       <c r="C69" s="24" t="n"/>
@@ -2782,7 +2766,7 @@
     </row>
     <row r="70">
       <c r="A70" s="22" t="n">
-        <v>46364</v>
+        <v>46366</v>
       </c>
       <c r="B70" s="23" t="n"/>
       <c r="C70" s="24" t="n"/>
@@ -2804,7 +2788,7 @@
     </row>
     <row r="71">
       <c r="A71" s="22" t="n">
-        <v>46365</v>
+        <v>46367</v>
       </c>
       <c r="B71" s="23" t="n"/>
       <c r="C71" s="24" t="n"/>
@@ -2826,7 +2810,7 @@
     </row>
     <row r="72">
       <c r="A72" s="22" t="n">
-        <v>46366</v>
+        <v>46368</v>
       </c>
       <c r="B72" s="23" t="n"/>
       <c r="C72" s="24" t="n"/>
@@ -2848,7 +2832,7 @@
     </row>
     <row r="73">
       <c r="A73" s="22" t="n">
-        <v>46367</v>
+        <v>46369</v>
       </c>
       <c r="B73" s="23" t="n"/>
       <c r="C73" s="24" t="n"/>
@@ -2870,7 +2854,7 @@
     </row>
     <row r="74">
       <c r="A74" s="22" t="n">
-        <v>46368</v>
+        <v>46370</v>
       </c>
       <c r="B74" s="23" t="n"/>
       <c r="C74" s="24" t="n"/>
@@ -2892,7 +2876,7 @@
     </row>
     <row r="75">
       <c r="A75" s="22" t="n">
-        <v>46369</v>
+        <v>46371</v>
       </c>
       <c r="B75" s="23" t="n"/>
       <c r="C75" s="24" t="n"/>
@@ -2914,7 +2898,7 @@
     </row>
     <row r="76">
       <c r="A76" s="22" t="n">
-        <v>46370</v>
+        <v>46372</v>
       </c>
       <c r="B76" s="23" t="n"/>
       <c r="C76" s="24" t="n"/>
@@ -2936,7 +2920,7 @@
     </row>
     <row r="77">
       <c r="A77" s="22" t="n">
-        <v>46371</v>
+        <v>46373</v>
       </c>
       <c r="B77" s="23" t="n"/>
       <c r="C77" s="24" t="n"/>
@@ -2958,7 +2942,7 @@
     </row>
     <row r="78">
       <c r="A78" s="22" t="n">
-        <v>46372</v>
+        <v>46374</v>
       </c>
       <c r="B78" s="23" t="n"/>
       <c r="C78" s="24" t="n"/>
@@ -2980,7 +2964,7 @@
     </row>
     <row r="79">
       <c r="A79" s="22" t="n">
-        <v>46373</v>
+        <v>46375</v>
       </c>
       <c r="B79" s="23" t="n"/>
       <c r="C79" s="24" t="n"/>
@@ -3002,7 +2986,7 @@
     </row>
     <row r="80">
       <c r="A80" s="22" t="n">
-        <v>46374</v>
+        <v>46376</v>
       </c>
       <c r="B80" s="23" t="n"/>
       <c r="C80" s="24" t="n"/>
@@ -3024,7 +3008,7 @@
     </row>
     <row r="81">
       <c r="A81" s="22" t="n">
-        <v>46375</v>
+        <v>46377</v>
       </c>
       <c r="B81" s="23" t="n"/>
       <c r="C81" s="24" t="n"/>
@@ -3046,7 +3030,7 @@
     </row>
     <row r="82">
       <c r="A82" s="22" t="n">
-        <v>46376</v>
+        <v>46378</v>
       </c>
       <c r="B82" s="23" t="n"/>
       <c r="C82" s="24" t="n"/>
@@ -3068,7 +3052,7 @@
     </row>
     <row r="83">
       <c r="A83" s="22" t="n">
-        <v>46377</v>
+        <v>46379</v>
       </c>
       <c r="B83" s="23" t="n"/>
       <c r="C83" s="24" t="n"/>
@@ -3090,7 +3074,7 @@
     </row>
     <row r="84">
       <c r="A84" s="22" t="n">
-        <v>46378</v>
+        <v>46380</v>
       </c>
       <c r="B84" s="23" t="n"/>
       <c r="C84" s="24" t="n"/>
@@ -3112,7 +3096,7 @@
     </row>
     <row r="85">
       <c r="A85" s="22" t="n">
-        <v>46379</v>
+        <v>46381</v>
       </c>
       <c r="B85" s="23" t="n"/>
       <c r="C85" s="24" t="n"/>
@@ -3134,7 +3118,7 @@
     </row>
     <row r="86">
       <c r="A86" s="22" t="n">
-        <v>46380</v>
+        <v>46382</v>
       </c>
       <c r="B86" s="23" t="n"/>
       <c r="C86" s="24" t="n"/>
@@ -3156,7 +3140,7 @@
     </row>
     <row r="87">
       <c r="A87" s="22" t="n">
-        <v>46381</v>
+        <v>46383</v>
       </c>
       <c r="B87" s="23" t="n"/>
       <c r="C87" s="24" t="n"/>
@@ -3178,7 +3162,7 @@
     </row>
     <row r="88">
       <c r="A88" s="22" t="n">
-        <v>46382</v>
+        <v>46384</v>
       </c>
       <c r="B88" s="23" t="n"/>
       <c r="C88" s="24" t="n"/>
@@ -3200,7 +3184,7 @@
     </row>
     <row r="89">
       <c r="A89" s="22" t="n">
-        <v>46383</v>
+        <v>46385</v>
       </c>
       <c r="B89" s="23" t="n"/>
       <c r="C89" s="24" t="n"/>
@@ -3222,7 +3206,7 @@
     </row>
     <row r="90">
       <c r="A90" s="22" t="n">
-        <v>46384</v>
+        <v>46386</v>
       </c>
       <c r="B90" s="23" t="n"/>
       <c r="C90" s="24" t="n"/>
@@ -3244,7 +3228,7 @@
     </row>
     <row r="91">
       <c r="A91" s="22" t="n">
-        <v>46385</v>
+        <v>46387</v>
       </c>
       <c r="B91" s="23" t="n"/>
       <c r="C91" s="24" t="n"/>
@@ -3265,84 +3249,40 @@
       <c r="I91" s="6" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="22" t="n">
-        <v>46386</v>
-      </c>
-      <c r="B92" s="23" t="n"/>
-      <c r="C92" s="24" t="n"/>
-      <c r="D92" s="24" t="n"/>
-      <c r="E92" s="24" t="n"/>
-      <c r="F92" s="25">
-        <f>IF(OR(B92="",E92="",E92=0),"",B92/E92)</f>
-        <v/>
-      </c>
-      <c r="G92" s="26">
-        <f>IF(OR(C92="",C92=0,D92=""),"",D92/C92)</f>
-        <v/>
-      </c>
-      <c r="H92" s="25">
-        <f>IF(B92="","",SUM($B$5:B92))</f>
-        <v/>
-      </c>
-      <c r="I92" s="6" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="22" t="n">
-        <v>46387</v>
-      </c>
-      <c r="B93" s="23" t="n"/>
-      <c r="C93" s="24" t="n"/>
-      <c r="D93" s="24" t="n"/>
-      <c r="E93" s="24" t="n"/>
-      <c r="F93" s="25">
-        <f>IF(OR(B93="",E93="",E93=0),"",B93/E93)</f>
-        <v/>
-      </c>
-      <c r="G93" s="26">
-        <f>IF(OR(C93="",C93=0,D93=""),"",D93/C93)</f>
-        <v/>
-      </c>
-      <c r="H93" s="25">
-        <f>IF(B93="","",SUM($B$5:B93))</f>
-        <v/>
-      </c>
-      <c r="I93" s="6" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="27" t="inlineStr">
+      <c r="A92" s="27" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B94" s="28">
-        <f>SUM(B5:B93)</f>
-        <v/>
-      </c>
-      <c r="C94" s="29">
-        <f>SUM(C5:C93)</f>
-        <v/>
-      </c>
-      <c r="D94" s="29">
-        <f>SUM(D5:D93)</f>
-        <v/>
-      </c>
-      <c r="E94" s="29">
-        <f>SUM(E5:E93)</f>
-        <v/>
-      </c>
-      <c r="F94" s="28">
-        <f>IFERROR(B94/E94,"")</f>
-        <v/>
-      </c>
-      <c r="G94" s="30">
-        <f>IFERROR(D94/C94,"")</f>
-        <v/>
-      </c>
-      <c r="H94" s="27" t="n"/>
-      <c r="I94" s="27" t="n"/>
+      <c r="B92" s="28">
+        <f>SUM(B5:B91)</f>
+        <v/>
+      </c>
+      <c r="C92" s="29">
+        <f>SUM(C5:C91)</f>
+        <v/>
+      </c>
+      <c r="D92" s="29">
+        <f>SUM(D5:D91)</f>
+        <v/>
+      </c>
+      <c r="E92" s="29">
+        <f>SUM(E5:E91)</f>
+        <v/>
+      </c>
+      <c r="F92" s="28">
+        <f>IFERROR(B92/E92,"")</f>
+        <v/>
+      </c>
+      <c r="G92" s="30">
+        <f>IFERROR(D92/C92,"")</f>
+        <v/>
+      </c>
+      <c r="H92" s="27" t="n"/>
+      <c r="I92" s="27" t="n"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F5:F93">
+  <conditionalFormatting sqref="F5:F91">
     <cfRule type="expression" priority="1" dxfId="1">
       <formula>AND(F5&lt;&gt;"",F5&lt;3)</formula>
     </cfRule>
@@ -7222,7 +7162,7 @@
         <v>46296</v>
       </c>
       <c r="B5" s="38">
-        <f>SUMIFS('Daily Ads'!$B$5:$B$93,'Daily Ads'!$A$5:$A$93,"&gt;="&amp;$A5,'Daily Ads'!$A$5:$A$93,"&lt;="&amp;EOMONTH($A5,0))</f>
+        <f>SUMIFS('Daily Ads'!$B$5:$B$91,'Daily Ads'!$A$5:$A$91,"&gt;="&amp;$A5,'Daily Ads'!$A$5:$A$91,"&lt;="&amp;EOMONTH($A5,0))</f>
         <v/>
       </c>
       <c r="C5" s="38">
@@ -7242,7 +7182,7 @@
         <v/>
       </c>
       <c r="G5" s="40">
-        <f>SUMIFS('Daily Ads'!$E$5:$E$93,'Daily Ads'!$A$5:$A$93,"&gt;="&amp;$A5,'Daily Ads'!$A$5:$A$93,"&lt;="&amp;EOMONTH($A5,0))</f>
+        <f>SUMIFS('Daily Ads'!$E$5:$E$91,'Daily Ads'!$A$5:$A$91,"&gt;="&amp;$A5,'Daily Ads'!$A$5:$A$91,"&lt;="&amp;EOMONTH($A5,0))</f>
         <v/>
       </c>
       <c r="H5" s="38">
@@ -7279,7 +7219,7 @@
         <v>46327</v>
       </c>
       <c r="B6" s="38">
-        <f>SUMIFS('Daily Ads'!$B$5:$B$93,'Daily Ads'!$A$5:$A$93,"&gt;="&amp;$A6,'Daily Ads'!$A$5:$A$93,"&lt;="&amp;EOMONTH($A6,0))</f>
+        <f>SUMIFS('Daily Ads'!$B$5:$B$91,'Daily Ads'!$A$5:$A$91,"&gt;="&amp;$A6,'Daily Ads'!$A$5:$A$91,"&lt;="&amp;EOMONTH($A6,0))</f>
         <v/>
       </c>
       <c r="C6" s="38">
@@ -7299,7 +7239,7 @@
         <v/>
       </c>
       <c r="G6" s="40">
-        <f>SUMIFS('Daily Ads'!$E$5:$E$93,'Daily Ads'!$A$5:$A$93,"&gt;="&amp;$A6,'Daily Ads'!$A$5:$A$93,"&lt;="&amp;EOMONTH($A6,0))</f>
+        <f>SUMIFS('Daily Ads'!$E$5:$E$91,'Daily Ads'!$A$5:$A$91,"&gt;="&amp;$A6,'Daily Ads'!$A$5:$A$91,"&lt;="&amp;EOMONTH($A6,0))</f>
         <v/>
       </c>
       <c r="H6" s="38">
@@ -7336,7 +7276,7 @@
         <v>46357</v>
       </c>
       <c r="B7" s="38">
-        <f>SUMIFS('Daily Ads'!$B$5:$B$93,'Daily Ads'!$A$5:$A$93,"&gt;="&amp;$A7,'Daily Ads'!$A$5:$A$93,"&lt;="&amp;EOMONTH($A7,0))</f>
+        <f>SUMIFS('Daily Ads'!$B$5:$B$91,'Daily Ads'!$A$5:$A$91,"&gt;="&amp;$A7,'Daily Ads'!$A$5:$A$91,"&lt;="&amp;EOMONTH($A7,0))</f>
         <v/>
       </c>
       <c r="C7" s="38">
@@ -7356,7 +7296,7 @@
         <v/>
       </c>
       <c r="G7" s="40">
-        <f>SUMIFS('Daily Ads'!$E$5:$E$93,'Daily Ads'!$A$5:$A$93,"&gt;="&amp;$A7,'Daily Ads'!$A$5:$A$93,"&lt;="&amp;EOMONTH($A7,0))</f>
+        <f>SUMIFS('Daily Ads'!$E$5:$E$91,'Daily Ads'!$A$5:$A$91,"&gt;="&amp;$A7,'Daily Ads'!$A$5:$A$91,"&lt;="&amp;EOMONTH($A7,0))</f>
         <v/>
       </c>
       <c r="H7" s="38">

</xml_diff>